<commit_message>
docs(showcase): show recording from the Test Explorer in the case study and screenshots
- Slide 4 and CASE_STUDY.md mention recording from the Test Explorer (Create & record,
  Record steps, Record a scenario).
- The capture script records the recorder clip from a scenario's "Record steps" button and adds
  an explorer-record screenshot; the throwaway scenario is deleted so samples are unchanged.
- Screenshots, clips, slides, PDF, Upwork and social images regenerated (sizes re-verified).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/run-report.xlsx
+++ b/docs/samples/run-report.xlsx
@@ -25,13 +25,13 @@
     <t>Environment</t>
   </si>
   <si>
-    <t>Local http://127.0.0.1:63437</t>
+    <t>Local http://127.0.0.1:55726</t>
   </si>
   <si>
     <t>Run</t>
   </si>
   <si>
-    <t>01M4A44QA78GH7GQJDK72S9SBP</t>
+    <t>01M4AKHGJMFZWYHCQ9FX46C4R4</t>
   </si>
   <si>
     <t>Status</t>
@@ -43,7 +43,7 @@
     <t>Started</t>
   </si>
   <si>
-    <t>2026-10-07T02:47:36.009Z</t>
+    <t>2026-10-07T07:16:43.734Z</t>
   </si>
   <si>
     <t>Duration (s)</t>
@@ -130,7 +130,7 @@
     <t>A JavaScript error broke the page: TypeError: Cannot read properties of undefined (reading 'name')</t>
   </si>
   <si>
-    <t>Fix the script error at at http://127.0.0.1:63437/:30:77.</t>
+    <t>Fix the script error at at http://127.0.0.1:55726/:30:77.</t>
   </si>
   <si>
     <t>Dashboard lists the next appointments</t>
@@ -274,10 +274,10 @@
     <t>Verify with the link in the email</t>
   </si>
   <si>
-    <t>Expected urlContains "verified=1", but got "http://127.0.0.1:63437/verfy?email=qa.link%2B01m4a44qa78gh7gqjdk72s9sbp%40example.test&amp;code=003052"</t>
-  </si>
-  <si>
-    <t>The page did not meet the check: Expected urlContains "verified=1", but got "http://127.0.0.1:63437/verfy?email=qa.link%2B01m4a44qa78gh7gqjdk72s9sbp%40example.test&amp;code=003052"</t>
+    <t>Expected urlContains "verified=1", but got "http://127.0.0.1:55726/verfy?email=qa.link%2B01m4akhgjmfzwyhcq9fx46c4r4%40example.test&amp;code=927456"</t>
+  </si>
+  <si>
+    <t>The page did not meet the check: Expected urlContains "verified=1", but got "http://127.0.0.1:55726/verfy?email=qa.link%2B01m4akhgjmfzwyhcq9fx46c4r4%40example.test&amp;code=927456"</t>
   </si>
   <si>
     <t>Compare the failure screenshot with the expectation.</t>
@@ -295,10 +295,10 @@
     <t>The doctors' schedule answers quickly</t>
   </si>
   <si>
-    <t>Expected time lt 150, but got 800</t>
-  </si>
-  <si>
-    <t>The API answered in 800 ms; the limit is 150 ms</t>
+    <t>Expected time lt 150, but got 785</t>
+  </si>
+  <si>
+    <t>The API answered in 785 ms; the limit is 150 ms</t>
   </si>
   <si>
     <t>Profile the endpoint: check its query plans and count its database queries; add an index or load related rows in one query.</t>
@@ -337,7 +337,7 @@
     <t>Open the login page</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:63437/login (200)</t>
+    <t>Opened http://127.0.0.1:55726/login (200)</t>
   </si>
   <si>
     <t>2</t>
@@ -412,7 +412,7 @@
     <t>A patient name</t>
   </si>
   <si>
-    <t>Generated name: Steve Runolfsdottir</t>
+    <t>Generated name: Edison Deckow</t>
   </si>
   <si>
     <t>Full name</t>
@@ -451,7 +451,7 @@
     <t>The patient page shows the name</t>
   </si>
   <si>
-    <t>Assert text "Steve Runolfsdottir"</t>
+    <t>Assert text "Edison Deckow"</t>
   </si>
   <si>
     <t>11</t>
@@ -466,7 +466,7 @@
     <t>Open the patient list</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:63437/patients (200)</t>
+    <t>Opened http://127.0.0.1:55726/patients (200)</t>
   </si>
   <si>
     <t>Search</t>
@@ -493,16 +493,16 @@
     <t>Log in as admin</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:63437/api/auth/login → 200 in 1 ms</t>
-  </si>
-  <si>
-    <t>Generated name: Jeremiah Smith</t>
+    <t>POST http://127.0.0.1:55726/api/auth/login → 200 in 1 ms</t>
+  </si>
+  <si>
+    <t>Generated name: Cleveland Kessler</t>
   </si>
   <si>
     <t>Register the patient</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:63437/api/patients → 201 in 1 ms</t>
+    <t>POST http://127.0.0.1:55726/api/patients → 201 in 1 ms</t>
   </si>
   <si>
     <t>Register the same patient again</t>
@@ -511,28 +511,28 @@
     <t>A free date</t>
   </si>
   <si>
-    <t>Generated date: 2032-05-31</t>
+    <t>Generated date: 2029-03-14</t>
   </si>
   <si>
     <t>Book a slot</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:63437/api/appointments → 201 in 1 ms</t>
+    <t>POST http://127.0.0.1:55726/api/appointments → 201 in 1 ms</t>
   </si>
   <si>
     <t>Book the same slot for another patient</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:63437/api/appointments → 409 in 0 ms</t>
+    <t>POST http://127.0.0.1:55726/api/appointments → 409 in 0 ms</t>
   </si>
   <si>
     <t>Open the booking form</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:63437/appointments/new (200)</t>
-  </si>
-  <si>
-    <t>Generated date: 2029-11-01</t>
+    <t>Opened http://127.0.0.1:55726/appointments/new (200)</t>
+  </si>
+  <si>
+    <t>Generated date: 2030-02-02</t>
   </si>
   <si>
     <t>Patient</t>
@@ -568,10 +568,10 @@
     <t>Listed</t>
   </si>
   <si>
-    <t>Assert textContains "2029-11-01"</t>
-  </si>
-  <si>
-    <t>Generated date: 2026-12-06</t>
+    <t>Assert textContains "2030-02-02"</t>
+  </si>
+  <si>
+    <t>Generated date: 2033-08-20</t>
   </si>
   <si>
     <t>Selected 2</t>
@@ -583,7 +583,7 @@
     <t>Selected 14:00</t>
   </si>
   <si>
-    <t>Generated date: 2028-10-25</t>
+    <t>Generated date: 2027-11-07</t>
   </si>
   <si>
     <t>Selected 11:00</t>
@@ -610,7 +610,7 @@
     <t>The second booking is refused</t>
   </si>
   <si>
-    <t>Generated date: 2028-07-23</t>
+    <t>Generated date: 2028-10-04</t>
   </si>
   <si>
     <t>Book Ana Lopez with Dr. Reyes</t>
@@ -640,16 +640,16 @@
     <t>GET /api/health</t>
   </si>
   <si>
-    <t>GET http://127.0.0.1:63437/api/health → 200 in 0 ms</t>
-  </si>
-  <si>
-    <t>Generated name: Hazel Mayert-Barrows</t>
+    <t>GET http://127.0.0.1:55726/api/health → 200 in 0 ms</t>
+  </si>
+  <si>
+    <t>Generated name: Libby Adams</t>
   </si>
   <si>
     <t>Create a patient</t>
   </si>
   <si>
-    <t>Generated date: 2027-07-13</t>
+    <t>Generated date: 2032-02-24</t>
   </si>
   <si>
     <t>Book an appointment for them</t>
@@ -658,7 +658,7 @@
     <t>Delete the patient</t>
   </si>
   <si>
-    <t>DELETE http://127.0.0.1:63437/api/patients/12 → 204 in 0 ms</t>
+    <t>DELETE http://127.0.0.1:55726/api/patients/12 → 204 in 0 ms</t>
   </si>
   <si>
     <t>No appointments are left for the deleted patient</t>
@@ -685,7 +685,7 @@
     <t>Open the sign-up page</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:63437/signup (200)</t>
+    <t>Opened http://127.0.0.1:55726/signup (200)</t>
   </si>
   <si>
     <t>Create the account</t>
@@ -706,7 +706,7 @@
     <t>Read the code</t>
   </si>
   <si>
-    <t>Extracted code 397560</t>
+    <t>Extracted code 367596</t>
   </si>
   <si>
     <t>Enter the code</t>
@@ -724,7 +724,7 @@
     <t>Open the link in the email</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:63437/verfy?email=qa.link%2B01m4a44qa78gh7gqjdk72s9sbp%40example.test&amp;code=003052 in the browser (404)</t>
+    <t>Opened http://127.0.0.1:55726/verfy?email=qa.link%2B01m4akhgjmfzwyhcq9fx46c4r4%40example.test&amp;code=927456 in the browser (404)</t>
   </si>
   <si>
     <t>Query plan of the patient lookup</t>
@@ -736,19 +736,19 @@
     <t>Web Vitals of the dashboard</t>
   </si>
   <si>
-    <t>http://127.0.0.1:63437/: LCP 16 ms, CLS 0, TTFB 3 ms, load 8 ms</t>
+    <t>http://127.0.0.1:55726/: LCP 16 ms, CLS 0, TTFB 3 ms, load 8 ms</t>
   </si>
   <si>
     <t>Doctors' schedule</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:63437/api/auth/login → 200 in 2 ms</t>
+    <t>POST http://127.0.0.1:55726/api/auth/login → 200 in 2 ms</t>
   </si>
   <si>
     <t>Visits report</t>
   </si>
   <si>
-    <t>Generated name: Mr. Jett Gulgowski</t>
+    <t>Generated name: Dion White</t>
   </si>
   <si>
     <t>Read the new patient code</t>
@@ -763,7 +763,7 @@
     <t>Find the patient through the API</t>
   </si>
   <si>
-    <t>GET http://127.0.0.1:63437/api/patients?q=PAT-1012 → 200 in 1 ms</t>
+    <t>GET http://127.0.0.1:55726/api/patients?q=PAT-1012 → 200 in 0 ms</t>
   </si>
   <si>
     <t>The row is in the database</t>
@@ -781,7 +781,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-10-07T02:49:38.234Z</t>
+    <t>2026-10-07T07:18:47.241Z</t>
   </si>
   <si>
     <t>Generated with</t>
@@ -1230,7 +1230,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>33.4</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1355,7 +1355,7 @@
         <v>30</v>
       </c>
       <c r="D2">
-        <v>1172</v>
+        <v>1153</v>
       </c>
       <c r="E2" t="s">
         <v>31</v>
@@ -1381,7 +1381,7 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E3" t="s">
         <v>31</v>
@@ -1407,7 +1407,7 @@
         <v>30</v>
       </c>
       <c r="D4">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E4" t="s">
         <v>31</v>
@@ -1433,7 +1433,7 @@
         <v>7</v>
       </c>
       <c r="D5">
-        <v>5864</v>
+        <v>5987</v>
       </c>
       <c r="E5" t="s">
         <v>36</v>
@@ -1459,7 +1459,7 @@
         <v>7</v>
       </c>
       <c r="D6">
-        <v>6076</v>
+        <v>6131</v>
       </c>
       <c r="E6" t="s">
         <v>40</v>
@@ -1485,7 +1485,7 @@
         <v>30</v>
       </c>
       <c r="D7">
-        <v>612</v>
+        <v>622</v>
       </c>
       <c r="E7" t="s">
         <v>31</v>
@@ -1511,7 +1511,7 @@
         <v>30</v>
       </c>
       <c r="D8">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E8" t="s">
         <v>31</v>
@@ -1537,7 +1537,7 @@
         <v>30</v>
       </c>
       <c r="D9">
-        <v>470</v>
+        <v>508</v>
       </c>
       <c r="E9" t="s">
         <v>31</v>
@@ -1563,7 +1563,7 @@
         <v>30</v>
       </c>
       <c r="D10">
-        <v>473</v>
+        <v>485</v>
       </c>
       <c r="E10" t="s">
         <v>31</v>
@@ -1589,7 +1589,7 @@
         <v>7</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="s">
         <v>47</v>
@@ -1641,7 +1641,7 @@
         <v>30</v>
       </c>
       <c r="D13">
-        <v>605</v>
+        <v>579</v>
       </c>
       <c r="E13" t="s">
         <v>31</v>
@@ -1667,7 +1667,7 @@
         <v>30</v>
       </c>
       <c r="D14">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="E14" t="s">
         <v>31</v>
@@ -1693,7 +1693,7 @@
         <v>7</v>
       </c>
       <c r="D15">
-        <v>6237</v>
+        <v>6331</v>
       </c>
       <c r="E15" t="s">
         <v>55</v>
@@ -1719,7 +1719,7 @@
         <v>7</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" t="s">
         <v>60</v>
@@ -1797,7 +1797,7 @@
         <v>7</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" t="s">
         <v>73</v>
@@ -1823,7 +1823,7 @@
         <v>30</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="s">
         <v>31</v>
@@ -1901,7 +1901,7 @@
         <v>30</v>
       </c>
       <c r="D23">
-        <v>461</v>
+        <v>482</v>
       </c>
       <c r="E23" t="s">
         <v>31</v>
@@ -1927,7 +1927,7 @@
         <v>7</v>
       </c>
       <c r="D24">
-        <v>5852</v>
+        <v>5846</v>
       </c>
       <c r="E24" t="s">
         <v>86</v>
@@ -1953,7 +1953,7 @@
         <v>30</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" t="s">
         <v>31</v>
@@ -1979,7 +1979,7 @@
         <v>30</v>
       </c>
       <c r="D26">
-        <v>756</v>
+        <v>739</v>
       </c>
       <c r="E26" t="s">
         <v>31</v>
@@ -2005,7 +2005,7 @@
         <v>7</v>
       </c>
       <c r="D27">
-        <v>802</v>
+        <v>788</v>
       </c>
       <c r="E27" t="s">
         <v>93</v>
@@ -2031,7 +2031,7 @@
         <v>7</v>
       </c>
       <c r="D28">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="E28" t="s">
         <v>97</v>
@@ -2057,7 +2057,7 @@
         <v>30</v>
       </c>
       <c r="D29">
-        <v>577</v>
+        <v>593</v>
       </c>
       <c r="E29" t="s">
         <v>31</v>
@@ -2126,7 +2126,7 @@
         <v>30</v>
       </c>
       <c r="E2">
-        <v>865</v>
+        <v>844</v>
       </c>
       <c r="F2" t="s">
         <v>107</v>
@@ -2146,7 +2146,7 @@
         <v>30</v>
       </c>
       <c r="E3">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F3" t="s">
         <v>31</v>
@@ -2166,7 +2166,7 @@
         <v>30</v>
       </c>
       <c r="E4">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F4" t="s">
         <v>31</v>
@@ -2206,7 +2206,7 @@
         <v>30</v>
       </c>
       <c r="E6">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F6" t="s">
         <v>114</v>
@@ -2226,7 +2226,7 @@
         <v>30</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F7" t="s">
         <v>117</v>
@@ -2246,7 +2246,7 @@
         <v>30</v>
       </c>
       <c r="E8">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
         <v>107</v>
@@ -2306,7 +2306,7 @@
         <v>30</v>
       </c>
       <c r="E11">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
         <v>31</v>
@@ -2346,7 +2346,7 @@
         <v>30</v>
       </c>
       <c r="E13">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F13" t="s">
         <v>117</v>
@@ -2366,7 +2366,7 @@
         <v>30</v>
       </c>
       <c r="E14">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F14" t="s">
         <v>118</v>
@@ -2386,7 +2386,7 @@
         <v>30</v>
       </c>
       <c r="E15">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F15" t="s">
         <v>107</v>
@@ -2426,7 +2426,7 @@
         <v>30</v>
       </c>
       <c r="E17">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F17" t="s">
         <v>31</v>
@@ -2446,7 +2446,7 @@
         <v>30</v>
       </c>
       <c r="E18">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F18" t="s">
         <v>31</v>
@@ -2466,7 +2466,7 @@
         <v>30</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F19" t="s">
         <v>125</v>
@@ -2486,7 +2486,7 @@
         <v>30</v>
       </c>
       <c r="E20">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F20" t="s">
         <v>127</v>
@@ -2506,7 +2506,7 @@
         <v>30</v>
       </c>
       <c r="E21">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F21" t="s">
         <v>118</v>
@@ -2526,7 +2526,7 @@
         <v>30</v>
       </c>
       <c r="E22">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F22" t="s">
         <v>107</v>
@@ -2586,7 +2586,7 @@
         <v>30</v>
       </c>
       <c r="E25">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F25" t="s">
         <v>31</v>
@@ -2606,7 +2606,7 @@
         <v>7</v>
       </c>
       <c r="E26">
-        <v>5096</v>
+        <v>5263</v>
       </c>
       <c r="F26" t="s">
         <v>36</v>
@@ -2646,7 +2646,7 @@
         <v>30</v>
       </c>
       <c r="E28">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F28" t="s">
         <v>107</v>
@@ -2686,7 +2686,7 @@
         <v>30</v>
       </c>
       <c r="E30">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F30" t="s">
         <v>31</v>
@@ -2706,7 +2706,7 @@
         <v>30</v>
       </c>
       <c r="E31">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F31" t="s">
         <v>31</v>
@@ -2726,7 +2726,7 @@
         <v>7</v>
       </c>
       <c r="E32">
-        <v>5281</v>
+        <v>5268</v>
       </c>
       <c r="F32" t="s">
         <v>40</v>
@@ -2746,7 +2746,7 @@
         <v>30</v>
       </c>
       <c r="E33">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="F33" t="s">
         <v>118</v>
@@ -2766,7 +2766,7 @@
         <v>30</v>
       </c>
       <c r="E34">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="F34" t="s">
         <v>107</v>
@@ -2786,7 +2786,7 @@
         <v>30</v>
       </c>
       <c r="E35">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F35" t="s">
         <v>31</v>
@@ -2846,7 +2846,7 @@
         <v>30</v>
       </c>
       <c r="E38">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F38" t="s">
         <v>31</v>
@@ -2886,7 +2886,7 @@
         <v>30</v>
       </c>
       <c r="E40">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F40" t="s">
         <v>31</v>
@@ -2946,7 +2946,7 @@
         <v>30</v>
       </c>
       <c r="E43">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F43" t="s">
         <v>31</v>
@@ -2966,7 +2966,7 @@
         <v>30</v>
       </c>
       <c r="E44">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F44" t="s">
         <v>31</v>
@@ -2986,7 +2986,7 @@
         <v>30</v>
       </c>
       <c r="E45">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F45" t="s">
         <v>142</v>
@@ -3026,7 +3026,7 @@
         <v>30</v>
       </c>
       <c r="E47">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F47" t="s">
         <v>148</v>
@@ -3106,7 +3106,7 @@
         <v>30</v>
       </c>
       <c r="E51">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F51" t="s">
         <v>31</v>
@@ -3126,7 +3126,7 @@
         <v>30</v>
       </c>
       <c r="E52">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F52" t="s">
         <v>31</v>
@@ -3146,7 +3146,7 @@
         <v>30</v>
       </c>
       <c r="E53">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F53" t="s">
         <v>150</v>
@@ -3166,7 +3166,7 @@
         <v>30</v>
       </c>
       <c r="E54">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F54" t="s">
         <v>31</v>
@@ -3186,7 +3186,7 @@
         <v>30</v>
       </c>
       <c r="E55">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F55" t="s">
         <v>31</v>
@@ -3206,7 +3206,7 @@
         <v>30</v>
       </c>
       <c r="E56">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F56" t="s">
         <v>153</v>
@@ -3226,7 +3226,7 @@
         <v>30</v>
       </c>
       <c r="E57">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F57" t="s">
         <v>118</v>
@@ -3246,7 +3246,7 @@
         <v>30</v>
       </c>
       <c r="E58">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F58" t="s">
         <v>107</v>
@@ -3266,7 +3266,7 @@
         <v>30</v>
       </c>
       <c r="E59">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F59" t="s">
         <v>31</v>
@@ -3286,7 +3286,7 @@
         <v>30</v>
       </c>
       <c r="E60">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F60" t="s">
         <v>31</v>
@@ -3306,7 +3306,7 @@
         <v>30</v>
       </c>
       <c r="E61">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F61" t="s">
         <v>31</v>
@@ -3326,7 +3326,7 @@
         <v>30</v>
       </c>
       <c r="E62">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F62" t="s">
         <v>150</v>
@@ -3346,7 +3346,7 @@
         <v>30</v>
       </c>
       <c r="E63">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="F63" t="s">
         <v>31</v>
@@ -3366,7 +3366,7 @@
         <v>30</v>
       </c>
       <c r="E64">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="F64" t="s">
         <v>31</v>
@@ -3386,7 +3386,7 @@
         <v>30</v>
       </c>
       <c r="E65">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F65" t="s">
         <v>154</v>
@@ -3406,7 +3406,7 @@
         <v>30</v>
       </c>
       <c r="E66">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="F66" t="s">
         <v>118</v>
@@ -3426,7 +3426,7 @@
         <v>30</v>
       </c>
       <c r="E67">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="F67" t="s">
         <v>107</v>
@@ -3446,7 +3446,7 @@
         <v>30</v>
       </c>
       <c r="E68">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F68" t="s">
         <v>31</v>
@@ -3466,7 +3466,7 @@
         <v>30</v>
       </c>
       <c r="E69">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F69" t="s">
         <v>31</v>
@@ -3486,7 +3486,7 @@
         <v>30</v>
       </c>
       <c r="E70">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F70" t="s">
         <v>31</v>
@@ -3526,7 +3526,7 @@
         <v>30</v>
       </c>
       <c r="E72">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F72" t="s">
         <v>31</v>
@@ -3546,7 +3546,7 @@
         <v>30</v>
       </c>
       <c r="E73">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="F73" t="s">
         <v>31</v>
@@ -3566,7 +3566,7 @@
         <v>30</v>
       </c>
       <c r="E74">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="F74" t="s">
         <v>155</v>
@@ -3666,7 +3666,7 @@
         <v>7</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F79" t="s">
         <v>47</v>
@@ -3786,7 +3786,7 @@
         <v>30</v>
       </c>
       <c r="E85">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="F85" t="s">
         <v>118</v>
@@ -3806,7 +3806,7 @@
         <v>30</v>
       </c>
       <c r="E86">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F86" t="s">
         <v>107</v>
@@ -3826,7 +3826,7 @@
         <v>30</v>
       </c>
       <c r="E87">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F87" t="s">
         <v>31</v>
@@ -3886,7 +3886,7 @@
         <v>30</v>
       </c>
       <c r="E90">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F90" t="s">
         <v>171</v>
@@ -3926,7 +3926,7 @@
         <v>30</v>
       </c>
       <c r="E92">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F92" t="s">
         <v>174</v>
@@ -3946,7 +3946,7 @@
         <v>30</v>
       </c>
       <c r="E93">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F93" t="s">
         <v>174</v>
@@ -3986,7 +3986,7 @@
         <v>30</v>
       </c>
       <c r="E95">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F95" t="s">
         <v>178</v>
@@ -4026,7 +4026,7 @@
         <v>30</v>
       </c>
       <c r="E97">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F97" t="s">
         <v>31</v>
@@ -4086,7 +4086,7 @@
         <v>30</v>
       </c>
       <c r="E100">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="F100" t="s">
         <v>118</v>
@@ -4106,7 +4106,7 @@
         <v>30</v>
       </c>
       <c r="E101">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F101" t="s">
         <v>107</v>
@@ -4166,7 +4166,7 @@
         <v>30</v>
       </c>
       <c r="E104">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F104" t="s">
         <v>31</v>
@@ -4206,7 +4206,7 @@
         <v>30</v>
       </c>
       <c r="E106">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F106" t="s">
         <v>171</v>
@@ -4226,7 +4226,7 @@
         <v>30</v>
       </c>
       <c r="E107">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F107" t="s">
         <v>186</v>
@@ -4246,7 +4246,7 @@
         <v>30</v>
       </c>
       <c r="E108">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F108" t="s">
         <v>187</v>
@@ -4266,7 +4266,7 @@
         <v>30</v>
       </c>
       <c r="E109">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F109" t="s">
         <v>31</v>
@@ -4286,7 +4286,7 @@
         <v>30</v>
       </c>
       <c r="E110">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F110" t="s">
         <v>188</v>
@@ -4346,7 +4346,7 @@
         <v>30</v>
       </c>
       <c r="E113">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F113" t="s">
         <v>118</v>
@@ -4366,7 +4366,7 @@
         <v>30</v>
       </c>
       <c r="E114">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F114" t="s">
         <v>107</v>
@@ -4406,7 +4406,7 @@
         <v>30</v>
       </c>
       <c r="E116">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F116" t="s">
         <v>31</v>
@@ -4426,7 +4426,7 @@
         <v>30</v>
       </c>
       <c r="E117">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F117" t="s">
         <v>31</v>
@@ -4466,7 +4466,7 @@
         <v>30</v>
       </c>
       <c r="E119">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F119" t="s">
         <v>171</v>
@@ -4526,7 +4526,7 @@
         <v>30</v>
       </c>
       <c r="E122">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F122" t="s">
         <v>31</v>
@@ -4546,7 +4546,7 @@
         <v>30</v>
       </c>
       <c r="E123">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F123" t="s">
         <v>190</v>
@@ -4566,7 +4566,7 @@
         <v>30</v>
       </c>
       <c r="E124">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F124" t="s">
         <v>31</v>
@@ -4586,7 +4586,7 @@
         <v>30</v>
       </c>
       <c r="E125">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F125" t="s">
         <v>182</v>
@@ -4606,7 +4606,7 @@
         <v>30</v>
       </c>
       <c r="E126">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F126" t="s">
         <v>171</v>
@@ -4626,7 +4626,7 @@
         <v>30</v>
       </c>
       <c r="E127">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F127" t="s">
         <v>186</v>
@@ -4686,7 +4686,7 @@
         <v>30</v>
       </c>
       <c r="E130">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F130" t="s">
         <v>190</v>
@@ -4706,7 +4706,7 @@
         <v>30</v>
       </c>
       <c r="E131">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F131" t="s">
         <v>31</v>
@@ -4726,7 +4726,7 @@
         <v>7</v>
       </c>
       <c r="E132">
-        <v>5078</v>
+        <v>5070</v>
       </c>
       <c r="F132" t="s">
         <v>55</v>
@@ -4766,7 +4766,7 @@
         <v>30</v>
       </c>
       <c r="E134">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F134" t="s">
         <v>159</v>
@@ -4806,7 +4806,7 @@
         <v>30</v>
       </c>
       <c r="E136">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F136" t="s">
         <v>167</v>
@@ -5006,7 +5006,7 @@
         <v>30</v>
       </c>
       <c r="E146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F146" t="s">
         <v>208</v>
@@ -5126,7 +5126,7 @@
         <v>30</v>
       </c>
       <c r="E152">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F152" t="s">
         <v>167</v>
@@ -5146,7 +5146,7 @@
         <v>30</v>
       </c>
       <c r="E153">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F153" t="s">
         <v>214</v>
@@ -5246,7 +5246,7 @@
         <v>30</v>
       </c>
       <c r="E158">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="F158" t="s">
         <v>223</v>
@@ -5286,7 +5286,7 @@
         <v>30</v>
       </c>
       <c r="E160">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F160" t="s">
         <v>31</v>
@@ -5306,7 +5306,7 @@
         <v>30</v>
       </c>
       <c r="E161">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F161" t="s">
         <v>31</v>
@@ -5326,7 +5326,7 @@
         <v>30</v>
       </c>
       <c r="E162">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F162" t="s">
         <v>31</v>
@@ -5386,7 +5386,7 @@
         <v>30</v>
       </c>
       <c r="E165">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F165" t="s">
         <v>230</v>
@@ -5406,7 +5406,7 @@
         <v>30</v>
       </c>
       <c r="E166">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F166" t="s">
         <v>31</v>
@@ -5426,7 +5426,7 @@
         <v>30</v>
       </c>
       <c r="E167">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F167" t="s">
         <v>31</v>
@@ -5446,7 +5446,7 @@
         <v>30</v>
       </c>
       <c r="E168">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F168" t="s">
         <v>234</v>
@@ -5486,7 +5486,7 @@
         <v>30</v>
       </c>
       <c r="E170">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F170" t="s">
         <v>223</v>
@@ -5506,7 +5506,7 @@
         <v>30</v>
       </c>
       <c r="E171">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F171" t="s">
         <v>31</v>
@@ -5526,7 +5526,7 @@
         <v>30</v>
       </c>
       <c r="E172">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F172" t="s">
         <v>31</v>
@@ -5546,7 +5546,7 @@
         <v>30</v>
       </c>
       <c r="E173">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F173" t="s">
         <v>31</v>
@@ -5566,7 +5566,7 @@
         <v>30</v>
       </c>
       <c r="E174">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F174" t="s">
         <v>31</v>
@@ -5586,7 +5586,7 @@
         <v>30</v>
       </c>
       <c r="E175">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F175" t="s">
         <v>226</v>
@@ -5626,7 +5626,7 @@
         <v>7</v>
       </c>
       <c r="E177">
-        <v>5074</v>
+        <v>5060</v>
       </c>
       <c r="F177" t="s">
         <v>86</v>
@@ -5646,7 +5646,7 @@
         <v>30</v>
       </c>
       <c r="E178">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F178" t="s">
         <v>238</v>
@@ -5666,7 +5666,7 @@
         <v>30</v>
       </c>
       <c r="E179">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="F179" t="s">
         <v>118</v>
@@ -5686,7 +5686,7 @@
         <v>30</v>
       </c>
       <c r="E180">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="F180" t="s">
         <v>107</v>
@@ -5706,7 +5706,7 @@
         <v>30</v>
       </c>
       <c r="E181">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F181" t="s">
         <v>31</v>
@@ -5726,7 +5726,7 @@
         <v>30</v>
       </c>
       <c r="E182">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F182" t="s">
         <v>31</v>
@@ -5766,7 +5766,7 @@
         <v>30</v>
       </c>
       <c r="E184">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F184" t="s">
         <v>240</v>
@@ -5786,7 +5786,7 @@
         <v>30</v>
       </c>
       <c r="E185">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F185" t="s">
         <v>157</v>
@@ -5826,7 +5826,7 @@
         <v>7</v>
       </c>
       <c r="E187">
-        <v>800</v>
+        <v>786</v>
       </c>
       <c r="F187" t="s">
         <v>93</v>
@@ -5846,7 +5846,7 @@
         <v>30</v>
       </c>
       <c r="E188">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F188" t="s">
         <v>157</v>
@@ -5906,7 +5906,7 @@
         <v>30</v>
       </c>
       <c r="E191">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="F191" t="s">
         <v>118</v>
@@ -5926,7 +5926,7 @@
         <v>30</v>
       </c>
       <c r="E192">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F192" t="s">
         <v>107</v>
@@ -5966,7 +5966,7 @@
         <v>30</v>
       </c>
       <c r="E194">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F194" t="s">
         <v>31</v>
@@ -6006,7 +6006,7 @@
         <v>30</v>
       </c>
       <c r="E196">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="F196" t="s">
         <v>31</v>
@@ -6046,7 +6046,7 @@
         <v>30</v>
       </c>
       <c r="E198">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F198" t="s">
         <v>31</v>
@@ -6086,7 +6086,7 @@
         <v>30</v>
       </c>
       <c r="E200">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F200" t="s">
         <v>31</v>
@@ -6106,7 +6106,7 @@
         <v>30</v>
       </c>
       <c r="E201">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F201" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
docs(showcase): recapture with the recorder toolbar docked at the bottom
</commit_message>
<xml_diff>
--- a/docs/samples/run-report.xlsx
+++ b/docs/samples/run-report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="259">
   <si>
     <t>Application</t>
   </si>
@@ -25,13 +25,13 @@
     <t>Environment</t>
   </si>
   <si>
-    <t>Local http://127.0.0.1:55726</t>
+    <t>Local http://127.0.0.1:52101</t>
   </si>
   <si>
     <t>Run</t>
   </si>
   <si>
-    <t>01M4AKHGJMFZWYHCQ9FX46C4R4</t>
+    <t>01M4AWG809S19Y00C9M7GVBFZZ</t>
   </si>
   <si>
     <t>Status</t>
@@ -43,7 +43,7 @@
     <t>Started</t>
   </si>
   <si>
-    <t>2026-10-07T07:16:43.734Z</t>
+    <t>2026-10-07T09:53:19.371Z</t>
   </si>
   <si>
     <t>Duration (s)</t>
@@ -130,7 +130,7 @@
     <t>A JavaScript error broke the page: TypeError: Cannot read properties of undefined (reading 'name')</t>
   </si>
   <si>
-    <t>Fix the script error at at http://127.0.0.1:55726/:30:77.</t>
+    <t>Fix the script error at at http://127.0.0.1:52101/:30:77.</t>
   </si>
   <si>
     <t>Dashboard lists the next appointments</t>
@@ -274,10 +274,10 @@
     <t>Verify with the link in the email</t>
   </si>
   <si>
-    <t>Expected urlContains "verified=1", but got "http://127.0.0.1:55726/verfy?email=qa.link%2B01m4akhgjmfzwyhcq9fx46c4r4%40example.test&amp;code=927456"</t>
-  </si>
-  <si>
-    <t>The page did not meet the check: Expected urlContains "verified=1", but got "http://127.0.0.1:55726/verfy?email=qa.link%2B01m4akhgjmfzwyhcq9fx46c4r4%40example.test&amp;code=927456"</t>
+    <t>Expected urlContains "verified=1", but got "http://127.0.0.1:52101/verfy?email=qa.link%2B01m4awg809s19y00c9m7gvbfzz%40example.test&amp;code=090052"</t>
+  </si>
+  <si>
+    <t>The page did not meet the check: Expected urlContains "verified=1", but got "http://127.0.0.1:52101/verfy?email=qa.link%2B01m4awg809s19y00c9m7gvbfzz%40example.test&amp;code=090052"</t>
   </si>
   <si>
     <t>Compare the failure screenshot with the expectation.</t>
@@ -295,10 +295,10 @@
     <t>The doctors' schedule answers quickly</t>
   </si>
   <si>
-    <t>Expected time lt 150, but got 785</t>
-  </si>
-  <si>
-    <t>The API answered in 785 ms; the limit is 150 ms</t>
+    <t>Expected time lt 150, but got 799</t>
+  </si>
+  <si>
+    <t>The API answered in 799 ms; the limit is 150 ms</t>
   </si>
   <si>
     <t>Profile the endpoint: check its query plans and count its database queries; add an index or load related rows in one query.</t>
@@ -337,7 +337,7 @@
     <t>Open the login page</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:55726/login (200)</t>
+    <t>Opened http://127.0.0.1:52101/login (200)</t>
   </si>
   <si>
     <t>2</t>
@@ -412,7 +412,7 @@
     <t>A patient name</t>
   </si>
   <si>
-    <t>Generated name: Edison Deckow</t>
+    <t>Generated name: Eliane Bahringer</t>
   </si>
   <si>
     <t>Full name</t>
@@ -451,7 +451,7 @@
     <t>The patient page shows the name</t>
   </si>
   <si>
-    <t>Assert text "Edison Deckow"</t>
+    <t>Assert text "Eliane Bahringer"</t>
   </si>
   <si>
     <t>11</t>
@@ -466,7 +466,7 @@
     <t>Open the patient list</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:55726/patients (200)</t>
+    <t>Opened http://127.0.0.1:52101/patients (200)</t>
   </si>
   <si>
     <t>Search</t>
@@ -493,16 +493,16 @@
     <t>Log in as admin</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:55726/api/auth/login → 200 in 1 ms</t>
-  </si>
-  <si>
-    <t>Generated name: Cleveland Kessler</t>
+    <t>POST http://127.0.0.1:52101/api/auth/login → 200 in 1 ms</t>
+  </si>
+  <si>
+    <t>Generated name: Sidney Kunze</t>
   </si>
   <si>
     <t>Register the patient</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:55726/api/patients → 201 in 1 ms</t>
+    <t>POST http://127.0.0.1:52101/api/patients → 201 in 1 ms</t>
   </si>
   <si>
     <t>Register the same patient again</t>
@@ -511,28 +511,28 @@
     <t>A free date</t>
   </si>
   <si>
-    <t>Generated date: 2029-03-14</t>
+    <t>Generated date: 2027-06-16</t>
   </si>
   <si>
     <t>Book a slot</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:55726/api/appointments → 201 in 1 ms</t>
+    <t>POST http://127.0.0.1:52101/api/appointments → 201 in 1 ms</t>
   </si>
   <si>
     <t>Book the same slot for another patient</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:55726/api/appointments → 409 in 0 ms</t>
+    <t>POST http://127.0.0.1:52101/api/appointments → 409 in 1 ms</t>
   </si>
   <si>
     <t>Open the booking form</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:55726/appointments/new (200)</t>
-  </si>
-  <si>
-    <t>Generated date: 2030-02-02</t>
+    <t>Opened http://127.0.0.1:52101/appointments/new (200)</t>
+  </si>
+  <si>
+    <t>Generated date: 2029-06-13</t>
   </si>
   <si>
     <t>Patient</t>
@@ -568,10 +568,10 @@
     <t>Listed</t>
   </si>
   <si>
-    <t>Assert textContains "2030-02-02"</t>
-  </si>
-  <si>
-    <t>Generated date: 2033-08-20</t>
+    <t>Assert textContains "2029-06-13"</t>
+  </si>
+  <si>
+    <t>Generated date: 2032-12-14</t>
   </si>
   <si>
     <t>Selected 2</t>
@@ -583,7 +583,7 @@
     <t>Selected 14:00</t>
   </si>
   <si>
-    <t>Generated date: 2027-11-07</t>
+    <t>Generated date: 2029-08-24</t>
   </si>
   <si>
     <t>Selected 11:00</t>
@@ -610,7 +610,7 @@
     <t>The second booking is refused</t>
   </si>
   <si>
-    <t>Generated date: 2028-10-04</t>
+    <t>Generated date: 2030-03-13</t>
   </si>
   <si>
     <t>Book Ana Lopez with Dr. Reyes</t>
@@ -640,16 +640,16 @@
     <t>GET /api/health</t>
   </si>
   <si>
-    <t>GET http://127.0.0.1:55726/api/health → 200 in 0 ms</t>
-  </si>
-  <si>
-    <t>Generated name: Libby Adams</t>
+    <t>GET http://127.0.0.1:52101/api/health → 200 in 1 ms</t>
+  </si>
+  <si>
+    <t>Generated name: Dr. Maryam Stanton</t>
   </si>
   <si>
     <t>Create a patient</t>
   </si>
   <si>
-    <t>Generated date: 2032-02-24</t>
+    <t>Generated date: 2033-12-05</t>
   </si>
   <si>
     <t>Book an appointment for them</t>
@@ -658,7 +658,7 @@
     <t>Delete the patient</t>
   </si>
   <si>
-    <t>DELETE http://127.0.0.1:55726/api/patients/12 → 204 in 0 ms</t>
+    <t>DELETE http://127.0.0.1:52101/api/patients/12 → 204 in 0 ms</t>
   </si>
   <si>
     <t>No appointments are left for the deleted patient</t>
@@ -685,7 +685,7 @@
     <t>Open the sign-up page</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:55726/signup (200)</t>
+    <t>Opened http://127.0.0.1:52101/signup (200)</t>
   </si>
   <si>
     <t>Create the account</t>
@@ -706,7 +706,7 @@
     <t>Read the code</t>
   </si>
   <si>
-    <t>Extracted code 367596</t>
+    <t>Extracted code 816900</t>
   </si>
   <si>
     <t>Enter the code</t>
@@ -724,7 +724,7 @@
     <t>Open the link in the email</t>
   </si>
   <si>
-    <t>Opened http://127.0.0.1:55726/verfy?email=qa.link%2B01m4akhgjmfzwyhcq9fx46c4r4%40example.test&amp;code=927456 in the browser (404)</t>
+    <t>Opened http://127.0.0.1:52101/verfy?email=qa.link%2B01m4awg809s19y00c9m7gvbfzz%40example.test&amp;code=090052 in the browser (404)</t>
   </si>
   <si>
     <t>Query plan of the patient lookup</t>
@@ -736,19 +736,22 @@
     <t>Web Vitals of the dashboard</t>
   </si>
   <si>
-    <t>http://127.0.0.1:55726/: LCP 16 ms, CLS 0, TTFB 3 ms, load 8 ms</t>
+    <t>http://127.0.0.1:52101/: LCP 16 ms, CLS 0, TTFB 3 ms, load 7 ms</t>
+  </si>
+  <si>
+    <t>POST http://127.0.0.1:52101/api/auth/login → 200 in 2 ms</t>
   </si>
   <si>
     <t>Doctors' schedule</t>
   </si>
   <si>
-    <t>POST http://127.0.0.1:55726/api/auth/login → 200 in 2 ms</t>
+    <t>POST http://127.0.0.1:52101/api/auth/login → 200 in 3 ms</t>
   </si>
   <si>
     <t>Visits report</t>
   </si>
   <si>
-    <t>Generated name: Dion White</t>
+    <t>Generated name: Alexander Cummings Sr.</t>
   </si>
   <si>
     <t>Read the new patient code</t>
@@ -763,7 +766,7 @@
     <t>Find the patient through the API</t>
   </si>
   <si>
-    <t>GET http://127.0.0.1:55726/api/patients?q=PAT-1012 → 200 in 0 ms</t>
+    <t>GET http://127.0.0.1:52101/api/patients?q=PAT-1012 → 200 in 1 ms</t>
   </si>
   <si>
     <t>The row is in the database</t>
@@ -781,7 +784,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-10-07T07:18:47.241Z</t>
+    <t>2026-10-07T09:55:25.137Z</t>
   </si>
   <si>
     <t>Generated with</t>
@@ -1230,7 +1233,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>33.7</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1355,7 +1358,7 @@
         <v>30</v>
       </c>
       <c r="D2">
-        <v>1153</v>
+        <v>1091</v>
       </c>
       <c r="E2" t="s">
         <v>31</v>
@@ -1381,7 +1384,7 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="E3" t="s">
         <v>31</v>
@@ -1407,7 +1410,7 @@
         <v>30</v>
       </c>
       <c r="D4">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="E4" t="s">
         <v>31</v>
@@ -1433,7 +1436,7 @@
         <v>7</v>
       </c>
       <c r="D5">
-        <v>5987</v>
+        <v>6016</v>
       </c>
       <c r="E5" t="s">
         <v>36</v>
@@ -1459,7 +1462,7 @@
         <v>7</v>
       </c>
       <c r="D6">
-        <v>6131</v>
+        <v>5908</v>
       </c>
       <c r="E6" t="s">
         <v>40</v>
@@ -1511,7 +1514,7 @@
         <v>30</v>
       </c>
       <c r="D8">
-        <v>460</v>
+        <v>479</v>
       </c>
       <c r="E8" t="s">
         <v>31</v>
@@ -1537,7 +1540,7 @@
         <v>30</v>
       </c>
       <c r="D9">
-        <v>508</v>
+        <v>461</v>
       </c>
       <c r="E9" t="s">
         <v>31</v>
@@ -1563,7 +1566,7 @@
         <v>30</v>
       </c>
       <c r="D10">
-        <v>485</v>
+        <v>478</v>
       </c>
       <c r="E10" t="s">
         <v>31</v>
@@ -1589,7 +1592,7 @@
         <v>7</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11" t="s">
         <v>47</v>
@@ -1615,7 +1618,7 @@
         <v>30</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="s">
         <v>31</v>
@@ -1641,7 +1644,7 @@
         <v>30</v>
       </c>
       <c r="D13">
-        <v>579</v>
+        <v>665</v>
       </c>
       <c r="E13" t="s">
         <v>31</v>
@@ -1667,7 +1670,7 @@
         <v>30</v>
       </c>
       <c r="D14">
-        <v>576</v>
+        <v>583</v>
       </c>
       <c r="E14" t="s">
         <v>31</v>
@@ -1693,7 +1696,7 @@
         <v>7</v>
       </c>
       <c r="D15">
-        <v>6331</v>
+        <v>6306</v>
       </c>
       <c r="E15" t="s">
         <v>55</v>
@@ -1719,7 +1722,7 @@
         <v>7</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="s">
         <v>60</v>
@@ -1823,7 +1826,7 @@
         <v>30</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="s">
         <v>31</v>
@@ -1901,7 +1904,7 @@
         <v>30</v>
       </c>
       <c r="D23">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="E23" t="s">
         <v>31</v>
@@ -1927,7 +1930,7 @@
         <v>7</v>
       </c>
       <c r="D24">
-        <v>5846</v>
+        <v>5927</v>
       </c>
       <c r="E24" t="s">
         <v>86</v>
@@ -1979,7 +1982,7 @@
         <v>30</v>
       </c>
       <c r="D26">
-        <v>739</v>
+        <v>784</v>
       </c>
       <c r="E26" t="s">
         <v>31</v>
@@ -2005,7 +2008,7 @@
         <v>7</v>
       </c>
       <c r="D27">
-        <v>788</v>
+        <v>803</v>
       </c>
       <c r="E27" t="s">
         <v>93</v>
@@ -2031,7 +2034,7 @@
         <v>7</v>
       </c>
       <c r="D28">
-        <v>1507</v>
+        <v>1509</v>
       </c>
       <c r="E28" t="s">
         <v>97</v>
@@ -2057,7 +2060,7 @@
         <v>30</v>
       </c>
       <c r="D29">
-        <v>593</v>
+        <v>710</v>
       </c>
       <c r="E29" t="s">
         <v>31</v>
@@ -2126,7 +2129,7 @@
         <v>30</v>
       </c>
       <c r="E2">
-        <v>844</v>
+        <v>806</v>
       </c>
       <c r="F2" t="s">
         <v>107</v>
@@ -2146,7 +2149,7 @@
         <v>30</v>
       </c>
       <c r="E3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
         <v>31</v>
@@ -2186,7 +2189,7 @@
         <v>30</v>
       </c>
       <c r="E5">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
         <v>31</v>
@@ -2206,7 +2209,7 @@
         <v>30</v>
       </c>
       <c r="E6">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
         <v>114</v>
@@ -2246,7 +2249,7 @@
         <v>30</v>
       </c>
       <c r="E8">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F8" t="s">
         <v>107</v>
@@ -2266,7 +2269,7 @@
         <v>30</v>
       </c>
       <c r="E9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F9" t="s">
         <v>31</v>
@@ -2286,7 +2289,7 @@
         <v>30</v>
       </c>
       <c r="E10">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F10" t="s">
         <v>31</v>
@@ -2306,7 +2309,7 @@
         <v>30</v>
       </c>
       <c r="E11">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F11" t="s">
         <v>31</v>
@@ -2346,7 +2349,7 @@
         <v>30</v>
       </c>
       <c r="E13">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F13" t="s">
         <v>117</v>
@@ -2366,7 +2369,7 @@
         <v>30</v>
       </c>
       <c r="E14">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F14" t="s">
         <v>118</v>
@@ -2386,7 +2389,7 @@
         <v>30</v>
       </c>
       <c r="E15">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F15" t="s">
         <v>107</v>
@@ -2426,7 +2429,7 @@
         <v>30</v>
       </c>
       <c r="E17">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F17" t="s">
         <v>31</v>
@@ -2446,7 +2449,7 @@
         <v>30</v>
       </c>
       <c r="E18">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F18" t="s">
         <v>31</v>
@@ -2486,7 +2489,7 @@
         <v>30</v>
       </c>
       <c r="E20">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F20" t="s">
         <v>127</v>
@@ -2506,7 +2509,7 @@
         <v>30</v>
       </c>
       <c r="E21">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F21" t="s">
         <v>118</v>
@@ -2526,7 +2529,7 @@
         <v>30</v>
       </c>
       <c r="E22">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F22" t="s">
         <v>107</v>
@@ -2546,7 +2549,7 @@
         <v>30</v>
       </c>
       <c r="E23">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F23" t="s">
         <v>31</v>
@@ -2606,7 +2609,7 @@
         <v>7</v>
       </c>
       <c r="E26">
-        <v>5263</v>
+        <v>5187</v>
       </c>
       <c r="F26" t="s">
         <v>36</v>
@@ -2626,7 +2629,7 @@
         <v>30</v>
       </c>
       <c r="E27">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="F27" t="s">
         <v>118</v>
@@ -2646,7 +2649,7 @@
         <v>30</v>
       </c>
       <c r="E28">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F28" t="s">
         <v>107</v>
@@ -2706,7 +2709,7 @@
         <v>30</v>
       </c>
       <c r="E31">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F31" t="s">
         <v>31</v>
@@ -2726,7 +2729,7 @@
         <v>7</v>
       </c>
       <c r="E32">
-        <v>5268</v>
+        <v>5134</v>
       </c>
       <c r="F32" t="s">
         <v>40</v>
@@ -2746,7 +2749,7 @@
         <v>30</v>
       </c>
       <c r="E33">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="F33" t="s">
         <v>118</v>
@@ -2766,7 +2769,7 @@
         <v>30</v>
       </c>
       <c r="E34">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F34" t="s">
         <v>107</v>
@@ -2786,7 +2789,7 @@
         <v>30</v>
       </c>
       <c r="E35">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F35" t="s">
         <v>31</v>
@@ -2826,7 +2829,7 @@
         <v>30</v>
       </c>
       <c r="E37">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F37" t="s">
         <v>31</v>
@@ -2846,7 +2849,7 @@
         <v>30</v>
       </c>
       <c r="E38">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F38" t="s">
         <v>31</v>
@@ -2866,7 +2869,7 @@
         <v>30</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="s">
         <v>132</v>
@@ -2906,7 +2909,7 @@
         <v>30</v>
       </c>
       <c r="E41">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F41" t="s">
         <v>31</v>
@@ -2926,7 +2929,7 @@
         <v>30</v>
       </c>
       <c r="E42">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F42" t="s">
         <v>31</v>
@@ -2966,7 +2969,7 @@
         <v>30</v>
       </c>
       <c r="E44">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F44" t="s">
         <v>31</v>
@@ -2986,7 +2989,7 @@
         <v>30</v>
       </c>
       <c r="E45">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F45" t="s">
         <v>142</v>
@@ -3006,7 +3009,7 @@
         <v>30</v>
       </c>
       <c r="E46">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F46" t="s">
         <v>145</v>
@@ -3026,7 +3029,7 @@
         <v>30</v>
       </c>
       <c r="E47">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
         <v>148</v>
@@ -3046,7 +3049,7 @@
         <v>30</v>
       </c>
       <c r="E48">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="F48" t="s">
         <v>118</v>
@@ -3066,7 +3069,7 @@
         <v>30</v>
       </c>
       <c r="E49">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="F49" t="s">
         <v>107</v>
@@ -3086,7 +3089,7 @@
         <v>30</v>
       </c>
       <c r="E50">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F50" t="s">
         <v>31</v>
@@ -3126,7 +3129,7 @@
         <v>30</v>
       </c>
       <c r="E52">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F52" t="s">
         <v>31</v>
@@ -3146,7 +3149,7 @@
         <v>30</v>
       </c>
       <c r="E53">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F53" t="s">
         <v>150</v>
@@ -3186,7 +3189,7 @@
         <v>30</v>
       </c>
       <c r="E55">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F55" t="s">
         <v>31</v>
@@ -3226,7 +3229,7 @@
         <v>30</v>
       </c>
       <c r="E57">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F57" t="s">
         <v>118</v>
@@ -3246,7 +3249,7 @@
         <v>30</v>
       </c>
       <c r="E58">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F58" t="s">
         <v>107</v>
@@ -3266,7 +3269,7 @@
         <v>30</v>
       </c>
       <c r="E59">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F59" t="s">
         <v>31</v>
@@ -3306,7 +3309,7 @@
         <v>30</v>
       </c>
       <c r="E61">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F61" t="s">
         <v>31</v>
@@ -3326,7 +3329,7 @@
         <v>30</v>
       </c>
       <c r="E62">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F62" t="s">
         <v>150</v>
@@ -3346,7 +3349,7 @@
         <v>30</v>
       </c>
       <c r="E63">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="F63" t="s">
         <v>31</v>
@@ -3366,7 +3369,7 @@
         <v>30</v>
       </c>
       <c r="E64">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="F64" t="s">
         <v>31</v>
@@ -3386,7 +3389,7 @@
         <v>30</v>
       </c>
       <c r="E65">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F65" t="s">
         <v>154</v>
@@ -3406,7 +3409,7 @@
         <v>30</v>
       </c>
       <c r="E66">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="F66" t="s">
         <v>118</v>
@@ -3426,7 +3429,7 @@
         <v>30</v>
       </c>
       <c r="E67">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="F67" t="s">
         <v>107</v>
@@ -3446,7 +3449,7 @@
         <v>30</v>
       </c>
       <c r="E68">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F68" t="s">
         <v>31</v>
@@ -3466,7 +3469,7 @@
         <v>30</v>
       </c>
       <c r="E69">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F69" t="s">
         <v>31</v>
@@ -3486,7 +3489,7 @@
         <v>30</v>
       </c>
       <c r="E70">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F70" t="s">
         <v>31</v>
@@ -3506,7 +3509,7 @@
         <v>30</v>
       </c>
       <c r="E71">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F71" t="s">
         <v>150</v>
@@ -3546,7 +3549,7 @@
         <v>30</v>
       </c>
       <c r="E73">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="F73" t="s">
         <v>31</v>
@@ -3566,7 +3569,7 @@
         <v>30</v>
       </c>
       <c r="E74">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="F74" t="s">
         <v>155</v>
@@ -3646,7 +3649,7 @@
         <v>30</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F78" t="s">
         <v>162</v>
@@ -3666,7 +3669,7 @@
         <v>7</v>
       </c>
       <c r="E79">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F79" t="s">
         <v>47</v>
@@ -3686,7 +3689,7 @@
         <v>30</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F80" t="s">
         <v>157</v>
@@ -3746,7 +3749,7 @@
         <v>30</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F83" t="s">
         <v>167</v>
@@ -3766,7 +3769,7 @@
         <v>30</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F84" t="s">
         <v>169</v>
@@ -3786,7 +3789,7 @@
         <v>30</v>
       </c>
       <c r="E85">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F85" t="s">
         <v>118</v>
@@ -3806,7 +3809,7 @@
         <v>30</v>
       </c>
       <c r="E86">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F86" t="s">
         <v>107</v>
@@ -3826,7 +3829,7 @@
         <v>30</v>
       </c>
       <c r="E87">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F87" t="s">
         <v>31</v>
@@ -3846,7 +3849,7 @@
         <v>30</v>
       </c>
       <c r="E88">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F88" t="s">
         <v>31</v>
@@ -3866,7 +3869,7 @@
         <v>30</v>
       </c>
       <c r="E89">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F89" t="s">
         <v>31</v>
@@ -3886,7 +3889,7 @@
         <v>30</v>
       </c>
       <c r="E90">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F90" t="s">
         <v>171</v>
@@ -3926,7 +3929,7 @@
         <v>30</v>
       </c>
       <c r="E92">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F92" t="s">
         <v>174</v>
@@ -3946,7 +3949,7 @@
         <v>30</v>
       </c>
       <c r="E93">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F93" t="s">
         <v>174</v>
@@ -3966,7 +3969,7 @@
         <v>30</v>
       </c>
       <c r="E94">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="F94" t="s">
         <v>31</v>
@@ -3986,7 +3989,7 @@
         <v>30</v>
       </c>
       <c r="E95">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F95" t="s">
         <v>178</v>
@@ -4006,7 +4009,7 @@
         <v>30</v>
       </c>
       <c r="E96">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="F96" t="s">
         <v>31</v>
@@ -4026,7 +4029,7 @@
         <v>30</v>
       </c>
       <c r="E97">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F97" t="s">
         <v>31</v>
@@ -4046,7 +4049,7 @@
         <v>30</v>
       </c>
       <c r="E98">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F98" t="s">
         <v>182</v>
@@ -4066,7 +4069,7 @@
         <v>30</v>
       </c>
       <c r="E99">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F99" t="s">
         <v>184</v>
@@ -4086,7 +4089,7 @@
         <v>30</v>
       </c>
       <c r="E100">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F100" t="s">
         <v>118</v>
@@ -4106,7 +4109,7 @@
         <v>30</v>
       </c>
       <c r="E101">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F101" t="s">
         <v>107</v>
@@ -4206,7 +4209,7 @@
         <v>30</v>
       </c>
       <c r="E106">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F106" t="s">
         <v>171</v>
@@ -4226,7 +4229,7 @@
         <v>30</v>
       </c>
       <c r="E107">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F107" t="s">
         <v>186</v>
@@ -4246,7 +4249,7 @@
         <v>30</v>
       </c>
       <c r="E108">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F108" t="s">
         <v>187</v>
@@ -4286,7 +4289,7 @@
         <v>30</v>
       </c>
       <c r="E110">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F110" t="s">
         <v>188</v>
@@ -4326,7 +4329,7 @@
         <v>30</v>
       </c>
       <c r="E112">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F112" t="s">
         <v>182</v>
@@ -4346,7 +4349,7 @@
         <v>30</v>
       </c>
       <c r="E113">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F113" t="s">
         <v>118</v>
@@ -4366,7 +4369,7 @@
         <v>30</v>
       </c>
       <c r="E114">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F114" t="s">
         <v>107</v>
@@ -4406,7 +4409,7 @@
         <v>30</v>
       </c>
       <c r="E116">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F116" t="s">
         <v>31</v>
@@ -4426,7 +4429,7 @@
         <v>30</v>
       </c>
       <c r="E117">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F117" t="s">
         <v>31</v>
@@ -4466,7 +4469,7 @@
         <v>30</v>
       </c>
       <c r="E119">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F119" t="s">
         <v>171</v>
@@ -4526,7 +4529,7 @@
         <v>30</v>
       </c>
       <c r="E122">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F122" t="s">
         <v>31</v>
@@ -4546,7 +4549,7 @@
         <v>30</v>
       </c>
       <c r="E123">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F123" t="s">
         <v>190</v>
@@ -4566,7 +4569,7 @@
         <v>30</v>
       </c>
       <c r="E124">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F124" t="s">
         <v>31</v>
@@ -4606,7 +4609,7 @@
         <v>30</v>
       </c>
       <c r="E126">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F126" t="s">
         <v>171</v>
@@ -4626,7 +4629,7 @@
         <v>30</v>
       </c>
       <c r="E127">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F127" t="s">
         <v>186</v>
@@ -4646,7 +4649,7 @@
         <v>30</v>
       </c>
       <c r="E128">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F128" t="s">
         <v>186</v>
@@ -4706,7 +4709,7 @@
         <v>30</v>
       </c>
       <c r="E131">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="F131" t="s">
         <v>31</v>
@@ -4726,7 +4729,7 @@
         <v>7</v>
       </c>
       <c r="E132">
-        <v>5070</v>
+        <v>5081</v>
       </c>
       <c r="F132" t="s">
         <v>55</v>
@@ -4826,7 +4829,7 @@
         <v>7</v>
       </c>
       <c r="E137">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F137" t="s">
         <v>60</v>
@@ -4846,7 +4849,7 @@
         <v>7</v>
       </c>
       <c r="E138">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F138" t="s">
         <v>65</v>
@@ -4946,7 +4949,7 @@
         <v>30</v>
       </c>
       <c r="E143">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F143" t="s">
         <v>157</v>
@@ -5006,7 +5009,7 @@
         <v>30</v>
       </c>
       <c r="E146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F146" t="s">
         <v>208</v>
@@ -5246,7 +5249,7 @@
         <v>30</v>
       </c>
       <c r="E158">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="F158" t="s">
         <v>223</v>
@@ -5286,7 +5289,7 @@
         <v>30</v>
       </c>
       <c r="E160">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F160" t="s">
         <v>31</v>
@@ -5306,7 +5309,7 @@
         <v>30</v>
       </c>
       <c r="E161">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F161" t="s">
         <v>31</v>
@@ -5326,7 +5329,7 @@
         <v>30</v>
       </c>
       <c r="E162">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F162" t="s">
         <v>31</v>
@@ -5346,7 +5349,7 @@
         <v>30</v>
       </c>
       <c r="E163">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F163" t="s">
         <v>226</v>
@@ -5366,7 +5369,7 @@
         <v>30</v>
       </c>
       <c r="E164">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F164" t="s">
         <v>228</v>
@@ -5426,7 +5429,7 @@
         <v>30</v>
       </c>
       <c r="E167">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F167" t="s">
         <v>31</v>
@@ -5446,7 +5449,7 @@
         <v>30</v>
       </c>
       <c r="E168">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F168" t="s">
         <v>234</v>
@@ -5486,7 +5489,7 @@
         <v>30</v>
       </c>
       <c r="E170">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F170" t="s">
         <v>223</v>
@@ -5506,7 +5509,7 @@
         <v>30</v>
       </c>
       <c r="E171">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F171" t="s">
         <v>31</v>
@@ -5526,7 +5529,7 @@
         <v>30</v>
       </c>
       <c r="E172">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F172" t="s">
         <v>31</v>
@@ -5566,7 +5569,7 @@
         <v>30</v>
       </c>
       <c r="E174">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F174" t="s">
         <v>31</v>
@@ -5586,7 +5589,7 @@
         <v>30</v>
       </c>
       <c r="E175">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F175" t="s">
         <v>226</v>
@@ -5606,7 +5609,7 @@
         <v>30</v>
       </c>
       <c r="E176">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F176" t="s">
         <v>236</v>
@@ -5626,7 +5629,7 @@
         <v>7</v>
       </c>
       <c r="E177">
-        <v>5060</v>
+        <v>5090</v>
       </c>
       <c r="F177" t="s">
         <v>86</v>
@@ -5666,7 +5669,7 @@
         <v>30</v>
       </c>
       <c r="E179">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="F179" t="s">
         <v>118</v>
@@ -5686,7 +5689,7 @@
         <v>30</v>
       </c>
       <c r="E180">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="F180" t="s">
         <v>107</v>
@@ -5746,7 +5749,7 @@
         <v>30</v>
       </c>
       <c r="E183">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F183" t="s">
         <v>31</v>
@@ -5766,7 +5769,7 @@
         <v>30</v>
       </c>
       <c r="E184">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="F184" t="s">
         <v>240</v>
@@ -5786,7 +5789,7 @@
         <v>30</v>
       </c>
       <c r="E185">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F185" t="s">
         <v>157</v>
@@ -5806,10 +5809,10 @@
         <v>30</v>
       </c>
       <c r="E186">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F186" t="s">
-        <v>159</v>
+        <v>241</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
@@ -5820,13 +5823,13 @@
         <v>108</v>
       </c>
       <c r="C187" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D187" t="s">
         <v>7</v>
       </c>
       <c r="E187">
-        <v>786</v>
+        <v>800</v>
       </c>
       <c r="F187" t="s">
         <v>93</v>
@@ -5846,7 +5849,7 @@
         <v>30</v>
       </c>
       <c r="E188">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F188" t="s">
         <v>157</v>
@@ -5866,10 +5869,10 @@
         <v>30</v>
       </c>
       <c r="E189">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F189" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
@@ -5880,7 +5883,7 @@
         <v>108</v>
       </c>
       <c r="C190" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D190" t="s">
         <v>7</v>
@@ -5906,7 +5909,7 @@
         <v>30</v>
       </c>
       <c r="E191">
-        <v>245</v>
+        <v>311</v>
       </c>
       <c r="F191" t="s">
         <v>118</v>
@@ -5926,7 +5929,7 @@
         <v>30</v>
       </c>
       <c r="E192">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="F192" t="s">
         <v>107</v>
@@ -5946,7 +5949,7 @@
         <v>30</v>
       </c>
       <c r="E193">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="F193" t="s">
         <v>31</v>
@@ -5966,7 +5969,7 @@
         <v>30</v>
       </c>
       <c r="E194">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="F194" t="s">
         <v>31</v>
@@ -5986,7 +5989,7 @@
         <v>30</v>
       </c>
       <c r="E195">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="F195" t="s">
         <v>31</v>
@@ -6006,7 +6009,7 @@
         <v>30</v>
       </c>
       <c r="E196">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F196" t="s">
         <v>31</v>
@@ -6029,7 +6032,7 @@
         <v>0</v>
       </c>
       <c r="F197" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
@@ -6066,7 +6069,7 @@
         <v>30</v>
       </c>
       <c r="E199">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="F199" t="s">
         <v>31</v>
@@ -6086,7 +6089,7 @@
         <v>30</v>
       </c>
       <c r="E200">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F200" t="s">
         <v>31</v>
@@ -6106,7 +6109,7 @@
         <v>30</v>
       </c>
       <c r="E201">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F201" t="s">
         <v>31</v>
@@ -6120,7 +6123,7 @@
         <v>138</v>
       </c>
       <c r="C202" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D202" t="s">
         <v>30</v>
@@ -6129,7 +6132,7 @@
         <v>33</v>
       </c>
       <c r="F202" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
@@ -6157,7 +6160,7 @@
         <v>99</v>
       </c>
       <c r="B204" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C204" t="s">
         <v>158</v>
@@ -6180,16 +6183,16 @@
         <v>143</v>
       </c>
       <c r="C205" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D205" t="s">
         <v>30</v>
       </c>
       <c r="E205">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F205" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
@@ -6200,16 +6203,16 @@
         <v>146</v>
       </c>
       <c r="C206" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D206" t="s">
         <v>30</v>
       </c>
       <c r="E206">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F206" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -6230,10 +6233,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -6246,18 +6249,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>